<commit_message>
Update harmonization sampling rate terminology
</commit_message>
<xml_diff>
--- a/harmonized/Biosignal_schema.xlsx
+++ b/harmonized/Biosignal_schema.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DLAB06\Desktop\M3DT_schema_git\harmonized\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DLAB06\Desktop\M3DT-DLAB-Harmonized-PSG-Schema-git\harmonized\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F002756-A75C-4C6B-86C6-A65244B141C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D94B44C9-7E97-4E92-BDF9-76B316096365}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -611,7 +611,7 @@
     <t>Cannula Flow, CannulaFlow</t>
   </si>
   <si>
-    <t>Harmonization target rate (Hz)</t>
+    <t>Harmonization sampling rate (Hz)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -705,7 +705,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
@@ -720,6 +720,7 @@
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
@@ -729,10 +730,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -745,7 +742,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1083,7 +1080,7 @@
       </c>
     </row>
     <row r="2" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1104,7 +1101,7 @@
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A3" s="7"/>
+      <c r="A3" s="8"/>
       <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
@@ -1123,7 +1120,7 @@
       <c r="K3" s="2"/>
     </row>
     <row r="4" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
+      <c r="A4" s="8"/>
       <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
@@ -1148,7 +1145,7 @@
       <c r="K4" s="2"/>
     </row>
     <row r="5" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A5" s="7"/>
+      <c r="A5" s="8"/>
       <c r="B5" s="2" t="s">
         <v>15</v>
       </c>
@@ -1173,7 +1170,7 @@
       <c r="K5" s="2"/>
     </row>
     <row r="6" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
+      <c r="A6" s="8"/>
       <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
@@ -1192,7 +1189,7 @@
       <c r="K6" s="2"/>
     </row>
     <row r="7" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A7" s="7"/>
+      <c r="A7" s="8"/>
       <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
@@ -1211,7 +1208,7 @@
       <c r="K7" s="2"/>
     </row>
     <row r="8" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A8" s="7"/>
+      <c r="A8" s="8"/>
       <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
@@ -1236,7 +1233,7 @@
       <c r="K8" s="2"/>
     </row>
     <row r="9" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A9" s="7"/>
+      <c r="A9" s="8"/>
       <c r="B9" s="2" t="s">
         <v>25</v>
       </c>
@@ -1261,7 +1258,7 @@
       <c r="K9" s="2"/>
     </row>
     <row r="10" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
+      <c r="A10" s="8"/>
       <c r="B10" s="2" t="s">
         <v>173</v>
       </c>
@@ -1278,7 +1275,7 @@
       <c r="K10" s="2"/>
     </row>
     <row r="11" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A11" s="7"/>
+      <c r="A11" s="8"/>
       <c r="B11" s="2" t="s">
         <v>174</v>
       </c>
@@ -1295,7 +1292,7 @@
       <c r="K11" s="2"/>
     </row>
     <row r="12" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
+      <c r="A12" s="8"/>
       <c r="B12" s="2" t="s">
         <v>29</v>
       </c>
@@ -1314,7 +1311,7 @@
       </c>
     </row>
     <row r="13" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A13" s="7"/>
+      <c r="A13" s="8"/>
       <c r="B13" s="2" t="s">
         <v>31</v>
       </c>
@@ -1333,7 +1330,7 @@
       </c>
     </row>
     <row r="14" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
+      <c r="A14" s="8"/>
       <c r="B14" s="2" t="s">
         <v>33</v>
       </c>
@@ -1356,7 +1353,7 @@
       </c>
     </row>
     <row r="15" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A15" s="7"/>
+      <c r="A15" s="8"/>
       <c r="B15" s="2" t="s">
         <v>36</v>
       </c>
@@ -1379,7 +1376,7 @@
       <c r="K15" s="2"/>
     </row>
     <row r="16" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A16" s="7"/>
+      <c r="A16" s="8"/>
       <c r="B16" s="2" t="s">
         <v>39</v>
       </c>
@@ -1398,7 +1395,7 @@
       </c>
     </row>
     <row r="17" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A17" s="7"/>
+      <c r="A17" s="8"/>
       <c r="B17" s="2" t="s">
         <v>41</v>
       </c>
@@ -1419,7 +1416,7 @@
       </c>
     </row>
     <row r="18" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A18" s="7"/>
+      <c r="A18" s="8"/>
       <c r="B18" s="2" t="s">
         <v>43</v>
       </c>
@@ -1438,7 +1435,7 @@
       <c r="K18" s="2"/>
     </row>
     <row r="19" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A19" s="7"/>
+      <c r="A19" s="8"/>
       <c r="B19" s="2" t="s">
         <v>45</v>
       </c>
@@ -1457,7 +1454,7 @@
       </c>
     </row>
     <row r="20" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A20" s="7"/>
+      <c r="A20" s="8"/>
       <c r="B20" s="2" t="s">
         <v>47</v>
       </c>
@@ -1476,7 +1473,7 @@
       <c r="K20" s="2"/>
     </row>
     <row r="21" spans="1:11" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="8"/>
+      <c r="A21" s="9"/>
       <c r="B21" s="3" t="s">
         <v>49</v>
       </c>
@@ -1495,7 +1492,7 @@
       <c r="K21" s="3"/>
     </row>
     <row r="22" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="7" t="s">
         <v>51</v>
       </c>
       <c r="B22" s="2" t="s">
@@ -1530,7 +1527,7 @@
       </c>
     </row>
     <row r="23" spans="1:11" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="8"/>
+      <c r="A23" s="9"/>
       <c r="B23" s="3" t="s">
         <v>58</v>
       </c>
@@ -1563,7 +1560,7 @@
       </c>
     </row>
     <row r="24" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="7" t="s">
         <v>64</v>
       </c>
       <c r="B24" s="2" t="s">
@@ -1590,7 +1587,7 @@
       <c r="K24" s="2"/>
     </row>
     <row r="25" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A25" s="7"/>
+      <c r="A25" s="8"/>
       <c r="B25" s="2" t="s">
         <v>68</v>
       </c>
@@ -1615,7 +1612,7 @@
       <c r="K25" s="2"/>
     </row>
     <row r="26" spans="1:11" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="8"/>
+      <c r="A26" s="9"/>
       <c r="B26" s="3" t="s">
         <v>71</v>
       </c>
@@ -1640,7 +1637,7 @@
       </c>
     </row>
     <row r="27" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="7" t="s">
         <v>93</v>
       </c>
       <c r="B27" s="2" t="s">
@@ -1663,7 +1660,7 @@
       </c>
     </row>
     <row r="28" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A28" s="7"/>
+      <c r="A28" s="8"/>
       <c r="B28" s="2" t="s">
         <v>97</v>
       </c>
@@ -1688,7 +1685,7 @@
       <c r="K28" s="2"/>
     </row>
     <row r="29" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A29" s="7"/>
+      <c r="A29" s="8"/>
       <c r="B29" s="2" t="s">
         <v>102</v>
       </c>
@@ -1713,7 +1710,7 @@
       <c r="K29" s="2"/>
     </row>
     <row r="30" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A30" s="7"/>
+      <c r="A30" s="8"/>
       <c r="B30" s="2" t="s">
         <v>107</v>
       </c>
@@ -1734,7 +1731,7 @@
       <c r="K30" s="2"/>
     </row>
     <row r="31" spans="1:11" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="8"/>
+      <c r="A31" s="9"/>
       <c r="B31" s="3" t="s">
         <v>110</v>
       </c>
@@ -1755,7 +1752,7 @@
       <c r="K31" s="3"/>
     </row>
     <row r="32" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A32" s="6" t="s">
+      <c r="A32" s="7" t="s">
         <v>73</v>
       </c>
       <c r="B32" s="2" t="s">
@@ -1776,7 +1773,7 @@
       <c r="K32" s="2"/>
     </row>
     <row r="33" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A33" s="7"/>
+      <c r="A33" s="8"/>
       <c r="B33" s="2" t="s">
         <v>79</v>
       </c>
@@ -1795,7 +1792,7 @@
       <c r="K33" s="2"/>
     </row>
     <row r="34" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A34" s="7"/>
+      <c r="A34" s="8"/>
       <c r="B34" s="2" t="s">
         <v>85</v>
       </c>
@@ -1814,7 +1811,7 @@
       <c r="K34" s="2"/>
     </row>
     <row r="35" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A35" s="7"/>
+      <c r="A35" s="8"/>
       <c r="B35" s="2" t="s">
         <v>87</v>
       </c>
@@ -1833,7 +1830,7 @@
       <c r="K35" s="2"/>
     </row>
     <row r="36" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A36" s="7"/>
+      <c r="A36" s="8"/>
       <c r="B36" s="2" t="s">
         <v>74</v>
       </c>
@@ -1854,7 +1851,7 @@
       </c>
     </row>
     <row r="37" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A37" s="7"/>
+      <c r="A37" s="8"/>
       <c r="B37" s="2" t="s">
         <v>89</v>
       </c>
@@ -1871,7 +1868,7 @@
       <c r="K37" s="2"/>
     </row>
     <row r="38" spans="1:11" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="8"/>
+      <c r="A38" s="9"/>
       <c r="B38" s="3" t="s">
         <v>81</v>
       </c>
@@ -1888,13 +1885,13 @@
       <c r="K38" s="3"/>
     </row>
     <row r="39" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A39" s="11" t="s">
+      <c r="A39" s="10" t="s">
         <v>175</v>
       </c>
       <c r="B39" t="s">
         <v>176</v>
       </c>
-      <c r="C39" s="9">
+      <c r="C39" s="2">
         <v>64</v>
       </c>
       <c r="G39" t="s">
@@ -1902,7 +1899,7 @@
       </c>
     </row>
     <row r="40" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A40" s="12"/>
+      <c r="A40" s="11"/>
       <c r="B40" t="s">
         <v>177</v>
       </c>
@@ -1920,30 +1917,30 @@
       </c>
     </row>
     <row r="41" spans="1:11" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="13"/>
-      <c r="B41" s="10" t="s">
+      <c r="A41" s="12"/>
+      <c r="B41" s="6" t="s">
         <v>178</v>
       </c>
       <c r="C41" s="3">
         <v>64</v>
       </c>
-      <c r="D41" s="10"/>
-      <c r="E41" s="10"/>
-      <c r="F41" s="10" t="s">
+      <c r="D41" s="6"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="G41" s="10"/>
-      <c r="H41" s="10" t="s">
+      <c r="G41" s="6"/>
+      <c r="H41" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="I41" s="10"/>
-      <c r="J41" s="10" t="s">
+      <c r="I41" s="6"/>
+      <c r="J41" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="K41" s="10"/>
+      <c r="K41" s="6"/>
     </row>
     <row r="42" spans="1:11" ht="34.5" x14ac:dyDescent="0.3">
-      <c r="A42" s="6" t="s">
+      <c r="A42" s="7" t="s">
         <v>111</v>
       </c>
       <c r="B42" s="2" t="s">
@@ -1974,7 +1971,7 @@
       </c>
     </row>
     <row r="43" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A43" s="7"/>
+      <c r="A43" s="8"/>
       <c r="B43" s="2" t="s">
         <v>115</v>
       </c>
@@ -1995,7 +1992,7 @@
       <c r="K43" s="2"/>
     </row>
     <row r="44" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A44" s="7"/>
+      <c r="A44" s="8"/>
       <c r="B44" s="2" t="s">
         <v>117</v>
       </c>
@@ -2024,7 +2021,7 @@
       </c>
     </row>
     <row r="45" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A45" s="7"/>
+      <c r="A45" s="8"/>
       <c r="B45" s="2" t="s">
         <v>123</v>
       </c>
@@ -2043,7 +2040,7 @@
       <c r="K45" s="2"/>
     </row>
     <row r="46" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A46" s="7"/>
+      <c r="A46" s="8"/>
       <c r="B46" s="2" t="s">
         <v>125</v>
       </c>
@@ -2062,7 +2059,7 @@
       <c r="K46" s="2"/>
     </row>
     <row r="47" spans="1:11" ht="34.5" x14ac:dyDescent="0.3">
-      <c r="A47" s="7"/>
+      <c r="A47" s="8"/>
       <c r="B47" s="2" t="s">
         <v>185</v>
       </c>
@@ -2083,7 +2080,7 @@
       <c r="K47" s="2"/>
     </row>
     <row r="48" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A48" s="7"/>
+      <c r="A48" s="8"/>
       <c r="B48" s="2" t="s">
         <v>188</v>
       </c>
@@ -2102,7 +2099,7 @@
       </c>
     </row>
     <row r="49" spans="1:11" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="8"/>
+      <c r="A49" s="9"/>
       <c r="B49" s="3" t="s">
         <v>190</v>
       </c>
@@ -2121,7 +2118,7 @@
       </c>
     </row>
     <row r="50" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A50" s="14" t="s">
+      <c r="A50" s="13" t="s">
         <v>127</v>
       </c>
       <c r="B50" s="2" t="s">
@@ -2154,7 +2151,7 @@
       <c r="K50" s="2"/>
     </row>
     <row r="51" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A51" s="15"/>
+      <c r="A51" s="14"/>
       <c r="B51" s="2" t="s">
         <v>134</v>
       </c>
@@ -2185,28 +2182,28 @@
       <c r="K51" s="2"/>
     </row>
     <row r="52" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A52" s="15"/>
-      <c r="B52" s="9" t="s">
+      <c r="A52" s="14"/>
+      <c r="B52" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="C52" s="9">
+      <c r="C52" s="2">
         <v>32</v>
       </c>
-      <c r="D52" s="9" t="s">
+      <c r="D52" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="E52" s="9"/>
-      <c r="F52" s="9" t="s">
+      <c r="E52" s="2"/>
+      <c r="F52" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="G52" s="9"/>
-      <c r="H52" s="9"/>
-      <c r="I52" s="9"/>
-      <c r="J52" s="9"/>
-      <c r="K52" s="9"/>
+      <c r="G52" s="2"/>
+      <c r="H52" s="2"/>
+      <c r="I52" s="2"/>
+      <c r="J52" s="2"/>
+      <c r="K52" s="2"/>
     </row>
     <row r="53" spans="1:11" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="16"/>
+      <c r="A53" s="15"/>
       <c r="B53" s="3" t="s">
         <v>112</v>
       </c>
@@ -2231,7 +2228,7 @@
       </c>
     </row>
     <row r="54" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A54" s="6" t="s">
+      <c r="A54" s="7" t="s">
         <v>143</v>
       </c>
       <c r="B54" s="2" t="s">
@@ -2262,7 +2259,7 @@
       <c r="K54" s="2"/>
     </row>
     <row r="55" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A55" s="7"/>
+      <c r="A55" s="8"/>
       <c r="B55" s="2" t="s">
         <v>150</v>
       </c>
@@ -2285,7 +2282,7 @@
       <c r="K55" s="2"/>
     </row>
     <row r="56" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A56" s="7"/>
+      <c r="A56" s="8"/>
       <c r="B56" s="2" t="s">
         <v>153</v>
       </c>
@@ -2314,7 +2311,7 @@
       </c>
     </row>
     <row r="57" spans="1:11" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A57" s="7"/>
+      <c r="A57" s="8"/>
       <c r="B57" s="2" t="s">
         <v>155</v>
       </c>
@@ -2339,7 +2336,7 @@
       <c r="K57" s="2"/>
     </row>
     <row r="58" spans="1:11" ht="18" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="8"/>
+      <c r="A58" s="9"/>
       <c r="B58" s="3" t="s">
         <v>159</v>
       </c>

</xml_diff>